<commit_message>
Alinear con roles de CORE y fuentes reales de Gestión Académica
- Cuentas demo con roles del catálogo de CORE (ACADEMIC_ADMIN, FINANCE_ADMIN);
  los permisos analytics:* quedan como supuesto a confirmar con CORE.
- Cuatrimestres desde los períodos de G9 (GET /api/planificacion/periodos),
  con gateway HTTP directo y token de servicio cuando hay ACADEMIC_URL.
- Catálogo de eventos: se reemplazan teacher.* por el evento de resultado
  de G9 (academic.course-result.published.v1, nombre propuesto).
- Docs: PREGUNTAS-A-GRUPOS.md con el estado actual del Trello, EVENTOS.md,
  Postman, README, CLAUDE.md y flujo de datos (xlsx).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Flujo_de_Datos_Modulo_7_Analitica.xlsx
+++ b/docs/Flujo_de_Datos_Modulo_7_Analitica.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Flujo de Datos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flujo de Datos'!$A$4:$F$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flujo de Datos'!$A$4:$F$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -556,7 +556,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Req: {"email": "mgarcia@uade.edu.ar", "password": "********"} Res: {"accessToken": "eyJhbGciOiJSUzI1NiIsImtpZCI6...", "expiresIn": 900, "user": {"id": "5d1e7c2a-8f43-4b9e-a6d0-2c7f9e1b3a58", "email": "mgarcia@uade.edu.ar", "roles": ["ADMIN_STAFF"], "permissions": ["analytics:academic:read", "analytics:finance:read"], "status": "ACTIVE"}}</t>
+          <t>Req: {"email": "mgarcia@uade.edu.ar", "password": "********"} Res: {"accessToken": "eyJhbGciOiJSUzI1NiIsImtpZCI6...", "expiresIn": 900, "user": {"id": "5d1e7c2a-8f43-4b9e-a6d0-2c7f9e1b3a58", "email": "mgarcia@uade.edu.ar", "roles": ["ACADEMIC_ADMIN"], "permissions": ["wallet:read:self", "wallet:credit:self", "academic:manage", "analytics:academic:read"], "status": "ACTIVE"}}</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>{"id": "5d1e7c2a-8f43-4b9e-a6d0-2c7f9e1b3a58", "email": "mgarcia@uade.edu.ar", "roles": ["ADMIN_STAFF"], "permissions": ["analytics:academic:read", "analytics:finance:read"], "status": "ACTIVE"}</t>
+          <t>{"id": "5d1e7c2a-8f43-4b9e-a6d0-2c7f9e1b3a58", "email": "mgarcia@uade.edu.ar", "roles": ["ACADEMIC_ADMIN"], "permissions": ["wallet:read:self", "wallet:credit:self", "academic:manage", "analytics:academic:read"], "status": "ACTIVE"}</t>
         </is>
       </c>
     </row>
@@ -679,12 +679,12 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>X-User-Id: uuid · X-User-Roles: csv · X-User-Permissions: csv · X-Correlation-Id: uuid · Authorization: Bearer &lt;jwt&gt; (lo revalidamos con JWKS). Autorización: analytics:academic:read → tablero académico y estadísticas de eventos; analytics:finance:read → tablero financiero. Sin permiso: 403 problem+json.</t>
+          <t>Authorization: Bearer &lt;jwt original&gt; · X-User-Id: uuid · X-User-Roles: csv · X-User-Permissions: csv · X-User-Career-Ids: csv · X-Correlation-Id: uuid · X-Core-Timestamp · X-Core-Signature (HMAC del gateway). La autorización sale del JWT validado con JWKS, no de los headers (la firma del gateway no cubre roles ni permisos). Permisos: analytics:academic:read → tablero académico y estadísticas de eventos; analytics:finance:read → tablero financiero. Se piden a CORE para los roles ACADEMIC_ADMIN y FINANCE_ADMIN (CORE es dueño del catálogo de roles y permisos). Sin permiso: 403 problem+json.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>X-User-Id: 5d1e7c2a-8f43-4b9e-a6d0-2c7f9e1b3a58 · X-User-Roles: ADMIN_STAFF · X-User-Permissions: analytics:academic:read,analytics:finance:read · X-Correlation-Id: f501201b-00bc-4200-99e0-6883500854f1</t>
+          <t>X-User-Id: 5d1e7c2a-8f43-4b9e-a6d0-2c7f9e1b3a58 · X-User-Roles: ACADEMIC_ADMIN · X-User-Permissions: wallet:read:self,wallet:credit:self,academic:manage,analytics:academic:read · X-Correlation-Id: f501201b-00bc-4200-99e0-6883500854f1</t>
         </is>
       </c>
     </row>
@@ -770,7 +770,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Cola analytics.all-events.v1 (exchange uadenet.events.v1, routingKeys ["#"], deadLetter uadenet.dlx.v1, maxRetries 3) — pedida por PR a contracts/topology.yaml</t>
+          <t>Cola analytics.all-events.v1 (exchange uadenet.events.v1, routingKeys ["#"], deadLetter uadenet.dlx.v1, maxRetries 3) — se pide a G10 (dueño, nombre, eventTypes, entorno y responsable); alternativa: webhooks por eventType (POST /internal/v1/subscriptions)</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>data: {"userId": "uuid", "email": "string", "status": "PENDING_ACTIVATION | ACTIVE | SUSPENDED | DISABLED", "roles": ["STUDENT | TEACHER | ADMIN_IT | ADMIN_STAFF"], "permissions": ["string"]} — aviso de alta o cambio de una persona (docentes = roles TEACHER): invalida el cache de nombres. No se copian datos de personas; el nombre se consulta a Backoffice por REST.</t>
+          <t>data: {"userId": "uuid", "email": "string", "status": "PENDING_ACTIVATION | ACTIVE | SUSPENDED | DISABLED", "roles": ["STUDENT | TEACHER | ADMIN | LIBRARIAN | STORE_ADMIN | OPERATIONS_ADMIN | ACADEMIC_ADMIN | FINANCE_ADMIN | IT_ADMIN"], "permissions": ["string"]} — aviso de alta o cambio de una persona (docentes = roles TEACHER): invalida el cache de nombres. No se copian datos de personas; el nombre se consulta a Backoffice por REST.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>data: {"userId": "uuid", "reason": "string"} — marca al docente como inactivo en el directorio local (sigue apareciendo en el histórico).</t>
+          <t>data: {"userId": "uuid", "reason": "string"} — aviso de baja de una persona: invalida el cache de nombres. Sus resultados históricos se siguen mostrando.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Portal del Docente</t>
+          <t>Gestión Académica y Planificación</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -962,24 +962,24 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>teacher.exam-result.published.v1</t>
+          <t>academic.course-result.published.v1 (nombre propuesto, a registrar en el catálogo de CORE)</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>data: {"studentId": "uuid", "courseId": "uuid", "subjectId": "uuid", "examId": "uuid", "grade": "number", "result": "string", "publishedAt": "ISO 8601 UTC", "teacherId": "uuid (propuesto, opcional — a acordar con Portal Docente y CORE)", "termId": "uuid (propuesto, opcional — a acordar con Portal Docente y CORE)"} — tasa de aprobación por materia (subjectId) y por cuatrimestre; con teacherId, tasa de aprobación por docente. Valores de result y examen que define la aprobación: a confirmar con Portal Docente.</t>
+          <t>data: {"studentId": "uuid", "courseId": "id del curso", "subjectId": "id de la asignatura", "periodId": "id del período", "siteId": "uuid (backofficeSiteId de la sede)", "finalGrade": "number (0-10)", "status": "APROBADO | DESAPROBADO", "resultDate": "date"} — un evento por alumno y curso cada vez que se carga o corrige la nota final (hoy G9 lo publica como resultado.publicado en su propia cola; tiene que pasar a POST /internal/v1/events de CORE). Cada publicación lleva un eventId nuevo; nos quedamos con el último resultado por alumno y curso. Alimenta la tasa de aprobación por materia, por docente y por cuatrimestre.</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>data: {"studentId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "courseId": "7b3c9d10-2e4f-4a61-8c5d-9f0e1a2b3c4d", "subjectId": "a1c2e3f4-5b6d-4e7f-8a9b-0c1d2e3f4a5b", "examId": "0e9d8c7b-6a5f-4e3d-2c1b-0a9f8e7d6c5b", "grade": 8, "result": "APPROVED", "publishedAt": "2026-07-10T21:00:00.000Z", "teacherId": "5f0a8e21-4c7b-4d19-9a3e-61b2c8d7f034", "termId": "d4e5f6a7-b8c9-4d0e-9f1a-2b3c4d5e6f70"}</t>
+          <t>data: {"studentId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "courseId": "42", "subjectId": "15", "periodId": "8", "siteId": "3e9b0a12-55cc-4d77-9a01-6b2f8c4e1d90", "finalGrade": 8.0, "status": "APROBADO", "resultDate": "2026-09-30"}</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Portal del Docente</t>
+          <t>Gestión Académica y Planificación</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -994,17 +994,17 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>teacher.attendance.recorded.v1</t>
+          <t>academic.term-defined.v1</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>data: {"studentId": "uuid", "courseId": "uuid", "classDate": "date", "present": "boolean"} — cursos con actividad en el cuatrimestre vigente, insumo de «materias en curso» (falta el cruce courseId → subjectId, a acordar con Gestión Académica / Portal Docente).</t>
+          <t>data: {"termId": "uuid", "startDate": "date", "endDate": "date"} — cuatrimestre vigente y anteriores, si G9 lo publica (está en el catálogo de CORE). Mientras tanto se toma de GET /periodos.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>data: {"studentId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "courseId": "7b3c9d10-2e4f-4a61-8c5d-9f0e1a2b3c4d", "classDate": "2026-09-16", "present": true}</t>
+          <t>data: {"termId": "d4e5f6a7-b8c9-4d0e-9f1a-2b3c4d5e6f70", "startDate": "2026-08-01", "endDate": "2026-11-30"}</t>
         </is>
       </c>
     </row>
@@ -1021,22 +1021,22 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Message Queue</t>
+          <t>Restful API</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>academic.term-defined.v1</t>
+          <t>GET {ACADEMIC_URL}/api/planificacion/cursos?periodoId={id} — directo al backend de Gestión Académica con token de servicio de CORE</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>data: {"termId": "uuid", "startDate": "date", "endDate": "date"} — define el cuatrimestre vigente y los anteriores (filtro de período del tablero académico).</t>
+          <t>Res 200: [{"id": "number", "codigo": "string", "asignaturaId": "number", "periodoId": "number", "sedeId": "number", "sedeNombre": "string", "estado": "PLANIFICADO | EN_CURSO | FINALIZADO | CANCELADO", "cupoMaximo": "number", "inscriptosActivos": "number"}] — cursos del cuatrimestre. Materias en curso = asignaturaId distintas con estado EN_CURSO. IDs hoy numéricos (CORE pide UUID).</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>data: {"termId": "d4e5f6a7-b8c9-4d0e-9f1a-2b3c4d5e6f70", "startDate": "2026-08-10", "endDate": "2026-12-12"}</t>
+          <t>GET {ACADEMIC_URL}/api/planificacion/cursos?periodoId=8 Res: [{"id": 42, "codigo": "DDA2-001", "asignaturaId": 15, "periodoId": 8, "sedeId": 2, "sedeNombre": "Sede Centro", "estado": "EN_CURSO", "cupoMaximo": 45, "inscriptosActivos": 30}]</t>
         </is>
       </c>
     </row>
@@ -1058,24 +1058,24 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>GET {ACADEMIC_URL}/api/v1/... — asignaturas por plan y carreras, directo al backend de Gestión Académica con token de servicio (paths a confirmar)</t>
+          <t>GET {ACADEMIC_URL}/api/planificacion/cursos/{cursoId} — directo, con token de servicio de CORE</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Asignatura: {"id": "uuid", "codigo": "string", "nombre": "string", "planId": "uuid"} · Carrera: {"id": "uuid", "nombre": "string", "facultad": "string"} — código y nombre de la materia para el tablero, y facultad para la tendencia por facultad. Carga inicial y cache.</t>
+          <t>Res 200: {"curso": {"id": "number", "asignatura": {"id": "number", "codigo": "string", "nombre": "string"}, "periodo": {"id": "number", "anio": "number", "numero": "number"}, "sedeId": "number", "estado": "string"}, "docentes": [{"docenteId": "string (UUID de Backoffice)", "rol": "TITULAR | ADJUNTO | AUXILIAR"}]} — docentes de cada curso, para la tasa de aprobación por docente (cruce courseId del resultado → docente).</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Asignatura: {"id": "a1c2e3f4-5b6d-4e7f-8a9b-0c1d2e3f4a5b", "codigo": "INF-302", "nombre": "Desarrollo de Aplicaciones II", "planId": "b2c3d4e5-f6a7-4b8c-9d0e-1f2a3b4c5d6e"} · Carrera: {"id": "c3d4e5f6-a7b8-4c9d-0e1f-2a3b4c5d6e7f", "nombre": "Ingeniería en Informática", "facultad": "Facultad de Ingeniería"}</t>
+          <t>{"curso": {"id": 42, "asignatura": {"id": 15, "codigo": "DDA2-002", "nombre": "Desarrollo de Aplicaciones II"}, "periodo": {"id": 8, "anio": 2026, "numero": 2}, "sedeId": 2, "estado": "EN_CURSO"}, "docentes": [{"docenteId": "5f0a8e21-4c7b-4d19-9a3e-61b2c8d7f034", "rol": "TITULAR"}]}</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Biblioteca Universitaria</t>
+          <t>Gestión Académica y Planificación</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1085,29 +1085,29 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Message Queue</t>
+          <t>Restful API</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>library.penalty.applied.v1</t>
+          <t>GET {ACADEMIC_URL}/api/planificacion/periodos — directo, con token de servicio de CORE</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>data: {"userId": "uuid", "loanId": "uuid", "daysLate": "number", "amount": "string decimal", "currency": "ARS"} — multas aplicadas por mes (complementa el concepto LIBRARY_FINE de los agregados de CORE).</t>
+          <t>Res 200: [{"id": "number", "anio": "number", "numero": "1 | 2", "fechaInicio": "date", "fechaFin": "date"}] — cuatrimestres para el filtro del tablero académico. La etiqueta AAAA-NC se arma con anio y numero.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>data: {"userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "loanId": "c8ed9311-6a6b-40c6-a798-5066d290c13c", "daysLate": 8, "amount": "2500.00", "currency": "ARS"}</t>
+          <t>[{"id": 8, "anio": 2026, "numero": 2, "fechaInicio": "2026-08-01", "fechaFin": "2026-11-30"}]</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Sistema de Comedor</t>
+          <t>Gestión Académica y Planificación</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1117,29 +1117,29 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Message Queue</t>
+          <t>Restful API</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>dining.reservation.created.v1</t>
+          <t>GET {ACADEMIC_URL}/api/planificacion/sedes — directo, con token de servicio de CORE</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>data: {"reservationId": "uuid", "userId": "uuid", "siteId": "uuid", "slotAt": "ISO 8601 UTC", "amount": "string decimal", "currency": "ARS"} — facturación de comedores por sede, cantidad de tickets y ticket promedio. Guardamos reservationId → siteId/amount para cruzar cancelaciones y asistencias.</t>
+          <t>Res 200: [{"id": "number", "backofficeSiteId": "uuid", "nombre": "string"}] — traduce el sedeId local de los cursos al siteId de Backoffice, que es el que usa el filtro de sede.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>data: {"reservationId": "58df9fe3-4883-4dca-9d9f-4770c81543cf", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "siteId": "3e9b0a12-55cc-4d77-9a01-6b2f8c4e1d90", "slotAt": "2026-09-15T15:00:00.000Z", "amount": "1500.00", "currency": "ARS"}</t>
+          <t>[{"id": 2, "backofficeSiteId": "3e9b0a12-55cc-4d77-9a01-6b2f8c4e1d90", "nombre": "Sede Centro"}]</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Sistema de Comedor</t>
+          <t>Gestión Académica y Planificación</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -1149,29 +1149,29 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Message Queue</t>
+          <t>Restful API</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>dining.reservation.cancelled.v1</t>
+          <t>GET {ACADEMIC_URL}/api/academica/carreras · /carreras/{carreraId}/planes · /planes/{planId}/asignaturas — directo, con token de servicio de CORE</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>data: {"reservationId": "uuid", "userId": "uuid", "slotAt": "ISO 8601 UTC", "cancelledAt": "ISO 8601 UTC"} — descuenta la reserva de la facturación; sede y monto se resuelven por reservationId.</t>
+          <t>Carrera: {"id": "number", "codigo": "string", "nombre": "string", "facultad": "string"} · Asignatura: {"id": "number", "codigo": "string", "nombre": "string", "planId": "number"} — código y nombre de cada materia y facultad de su carrera (tendencia por facultad). Carga inicial y cache.</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>data: {"reservationId": "58df9fe3-4883-4dca-9d9f-4770c81543cf", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "slotAt": "2026-09-15T15:00:00.000Z", "cancelledAt": "2026-09-14T18:10:00.000Z"}</t>
+          <t>Carrera: {"id": 1, "codigo": "ING-001", "nombre": "Ingeniería en Informática", "facultad": "Facultad de Ingeniería"} · Asignatura: {"id": 15, "codigo": "DDA2-002", "nombre": "Desarrollo de Aplicaciones II", "planId": 3}</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Sistema de Comedor</t>
+          <t>Biblioteca Universitaria</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1186,24 +1186,24 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>dining.attendance.recorded.v1</t>
+          <t>library.penalty.applied.v1</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>data: {"reservationId": "uuid", "userId": "uuid", "attendedAt": "ISO 8601 UTC"} — asistencia a la reserva. El monto restituido se toma de core.wallet.transaction-reversed.v1 (concept REFUND).</t>
+          <t>data: {"userId": "uuid", "loanId": "uuid", "daysLate": "number", "amount": "string decimal", "currency": "ARS"} — multas aplicadas por mes (complementa el concepto LIBRARY_FINE de los agregados de CORE).</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>data: {"reservationId": "58df9fe3-4883-4dca-9d9f-4770c81543cf", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "attendedAt": "2026-09-15T15:05:00.000Z"}</t>
+          <t>data: {"userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "loanId": "c8ed9311-6a6b-40c6-a798-5066d290c13c", "daysLate": 8, "amount": "2500.00", "currency": "ARS"}</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Tienda del Campus</t>
+          <t>Sistema de Comedor</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -1218,24 +1218,24 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>store.purchase.completed.v1</t>
+          <t>dining.reservation.created.v1</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>data: {"purchaseId": "uuid", "userId": "uuid", "total": "string decimal", "currency": "ARS", "items": [{"productId": "uuid", "productName": "string (al momento de la compra)", "category": "string", "quantity": "number", "unitPrice": "string decimal", "subtotal": "string decimal"}], "siteId": "uuid (opcional)"} — productos más vendidos (unidades y facturación por producto). userId no se persiste. Campos de items[] a confirmar con Tienda.</t>
+          <t>data: {"reservationId": "uuid", "userId": "uuid", "siteId": "uuid", "slotAt": "ISO 8601 UTC", "amount": "string decimal", "currency": "ARS"} — facturación de comedores por sede, cantidad de tickets y ticket promedio. Guardamos reservationId → siteId/amount para cruzar cancelaciones y asistencias.</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>data: {"purchaseId": "93b28f67-e111-4a0d-b857-fdd015c4d3f1", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "total": "3500.00", "currency": "ARS", "items": [{"productId": "1a2b3c4d-5e6f-4a7b-8c9d-0e1f2a3b4c5d", "productName": "Buzo UADE azul", "category": "Indumentaria", "quantity": 1, "unitPrice": "3500.00", "subtotal": "3500.00"}], "siteId": "3e9b0a12-55cc-4d77-9a01-6b2f8c4e1d90"}</t>
+          <t>data: {"reservationId": "58df9fe3-4883-4dca-9d9f-4770c81543cf", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "siteId": "3e9b0a12-55cc-4d77-9a01-6b2f8c4e1d90", "slotAt": "2026-09-15T15:00:00.000Z", "amount": "1500.00", "currency": "ARS"}</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Eventos Académicos</t>
+          <t>Sistema de Comedor</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -1250,24 +1250,24 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>events.event.created.v1</t>
+          <t>dining.reservation.cancelled.v1</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>data: {"eventId": "uuid", "title": "string", "locationId": "uuid", "startAt": "ISO 8601 UTC", "endAt": "ISO 8601 UTC", "capacity": "number", "price": "string decimal | null", "currency": "ARS"} — frecuencia de eventos por mes y ocupación de cupo. La sede sale de locationId → siteId (backoffice.location.upserted.v1). Un evento cuenta como realizado cuando pasa endAt.</t>
+          <t>data: {"reservationId": "uuid", "userId": "uuid", "slotAt": "ISO 8601 UTC", "cancelledAt": "ISO 8601 UTC"} — descuenta la reserva de la facturación; sede y monto se resuelven por reservationId.</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>data: {"eventId": "65a783d1-d407-442d-8d09-a6d2abfe9321", "title": "Jornada de Ingeniería", "locationId": "c41a77b2-9e0d-4f36-8b21-77aa1c9de405", "startAt": "2026-10-12T21:00:00.000Z", "endAt": "2026-10-13T00:00:00.000Z", "capacity": 200, "price": "1800.00", "currency": "ARS"}</t>
+          <t>data: {"reservationId": "58df9fe3-4883-4dca-9d9f-4770c81543cf", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "slotAt": "2026-09-15T15:00:00.000Z", "cancelledAt": "2026-09-14T18:10:00.000Z"}</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Eventos Académicos</t>
+          <t>Sistema de Comedor</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1282,24 +1282,24 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>events.registration.completed.v1</t>
+          <t>dining.attendance.recorded.v1</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>data: {"eventId": "uuid", "registrationId": "uuid", "userId": "uuid", "amount": "string decimal", "currency": "ARS"} — inscriptos por evento e ingresos por inscripción paga (amount = "0.00" si es gratuito).</t>
+          <t>data: {"reservationId": "uuid", "userId": "uuid", "attendedAt": "ISO 8601 UTC"} — asistencia a la reserva. El monto restituido se toma de core.wallet.transaction-reversed.v1 (concept REFUND).</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>data: {"eventId": "65a783d1-d407-442d-8d09-a6d2abfe9321", "registrationId": "5e8d0b31-9c47-4a26-b18f-72e4c0d95a68", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "amount": "1800.00", "currency": "ARS"}</t>
+          <t>data: {"reservationId": "58df9fe3-4883-4dca-9d9f-4770c81543cf", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "attendedAt": "2026-09-15T15:05:00.000Z"}</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Eventos Académicos</t>
+          <t>Tienda del Campus</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -1314,24 +1314,24 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>events.attendance.recorded.v1</t>
+          <t>store.purchase.completed.v1</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>data: {"eventId": "uuid", "userId": "uuid", "present": "boolean", "checkedAt": "ISO 8601 UTC"} — concurrencia (presentes) y tasa de presentismo (presentes / inscriptos).</t>
+          <t>data: {"purchaseId": "uuid", "userId": "uuid", "total": "string decimal", "currency": "ARS", "items": [{"productId": "uuid", "productName": "string (al momento de la compra)", "category": "string", "quantity": "number", "unitPrice": "string decimal", "subtotal": "string decimal"}], "siteId": "uuid (opcional)"} — productos más vendidos (unidades y facturación por producto). userId no se persiste. Campos de items[] a confirmar con Tienda.</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>data: {"eventId": "65a783d1-d407-442d-8d09-a6d2abfe9321", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "present": true, "checkedAt": "2026-10-12T21:07:44.000Z"}</t>
+          <t>data: {"purchaseId": "93b28f67-e111-4a0d-b857-fdd015c4d3f1", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "total": "3500.00", "currency": "ARS", "items": [{"productId": "1a2b3c4d-5e6f-4a7b-8c9d-0e1f2a3b4c5d", "productName": "Buzo UADE azul", "category": "Indumentaria", "quantity": 1, "unitPrice": "3500.00", "subtotal": "3500.00"}], "siteId": "3e9b0a12-55cc-4d77-9a01-6b2f8c4e1d90"}</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>CORE (Wallet)</t>
+          <t>Eventos Académicos</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -1346,24 +1346,24 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>core.wallet.transaction-posted.v1</t>
+          <t>events.event.created.v1</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>data: {"transactionId": "uuid", "userId": "uuid", "type": "CREDIT | DEBIT | REVERSAL", "concept": "TOP_UP | PAYROLL | SCHOLARSHIP | ADJUSTMENT | LIBRARY_FINE | DINING_RESERVATION | STORE_PURCHASE | EVENT_REGISTRATION | REFUND", "amount": "string decimal", "currency": "ARS", "sourceModule": "string", "externalReference": "string", "status": "POSTED"} — movimientos del mes en curso por concepto (los totales oficiales salen de aggregates). No se persiste userId.</t>
+          <t>data: {"eventId": "uuid", "title": "string", "locationId": "uuid", "startAt": "ISO 8601 UTC", "endAt": "ISO 8601 UTC", "capacity": "number", "price": "string decimal | null", "currency": "ARS"} — frecuencia de eventos por mes y ocupación de cupo. La sede sale de locationId → siteId (backoffice.location.upserted.v1). Un evento cuenta como realizado cuando pasa endAt.</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>data: {"transactionId": "386865f7-c8aa-4aba-a374-ec9e6f8a6300", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "type": "DEBIT", "concept": "STORE_PURCHASE", "amount": "3500.00", "currency": "ARS", "sourceModule": "store", "externalReference": "purchase/93b28f67-e111-4a0d-b857-fdd015c4d3f1", "status": "POSTED"}</t>
+          <t>data: {"eventId": "65a783d1-d407-442d-8d09-a6d2abfe9321", "title": "Jornada de Ingeniería", "locationId": "c41a77b2-9e0d-4f36-8b21-77aa1c9de405", "startAt": "2026-10-12T21:00:00.000Z", "endAt": "2026-10-13T00:00:00.000Z", "capacity": 200, "price": "1800.00", "currency": "ARS"}</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>CORE (Wallet)</t>
+          <t>Eventos Académicos</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1378,24 +1378,24 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>core.wallet.transaction-rejected.v1</t>
+          <t>events.registration.completed.v1</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>data: {"userId": "uuid", "type": "string", "concept": "string", "amount": "string decimal", "currency": "ARS", "sourceModule": "string", "externalReference": "string", "reasonCode": "string"} — cobros rechazados por concepto (p. ej. saldo insuficiente). Informativo.</t>
+          <t>data: {"eventId": "uuid", "registrationId": "uuid", "userId": "uuid", "amount": "string decimal", "currency": "ARS"} — inscriptos por evento e ingresos por inscripción paga (amount = "0.00" si es gratuito).</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>data: {"userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "type": "DEBIT", "concept": "DINING_RESERVATION", "amount": "1500.00", "currency": "ARS", "sourceModule": "dining", "externalReference": "reservation/58df9fe3-4883-4dca-9d9f-4770c81543cf", "reasonCode": "WALLET_INSUFFICIENT_FUNDS"}</t>
+          <t>data: {"eventId": "65a783d1-d407-442d-8d09-a6d2abfe9321", "registrationId": "5e8d0b31-9c47-4a26-b18f-72e4c0d95a68", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "amount": "1800.00", "currency": "ARS"}</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>CORE (Wallet)</t>
+          <t>Eventos Académicos</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -1410,113 +1410,113 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>core.wallet.transaction-reversed.v1</t>
+          <t>events.attendance.recorded.v1</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>data: {"transactionId": "uuid", "originalTransactionId": "uuid", "userId": "uuid", "concept": "REFUND", "amount": "string decimal", "currency": "ARS"} — reintegros: restitución de reservas de comedor asistidas y reversas de cobros de Tienda y Eventos.</t>
+          <t>data: {"eventId": "uuid", "userId": "uuid", "present": "boolean", "checkedAt": "ISO 8601 UTC"} — concurrencia (presentes) y tasa de presentismo (presentes / inscriptos).</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>data: {"transactionId": "0c3b6d21-9a44-4f7d-b2e8-15ac9f3d7e60", "originalTransactionId": "386865f7-c8aa-4aba-a374-ec9e6f8a6300", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "concept": "REFUND", "amount": "1500.00", "currency": "ARS"}</t>
+          <t>data: {"eventId": "65a783d1-d407-442d-8d09-a6d2abfe9321", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "present": true, "checkedAt": "2026-10-12T21:07:44.000Z"}</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>— (consumo interno: portal de Analítica)</t>
+          <t>CORE (Wallet)</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Salida</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Restful API</t>
+          <t>Message Queue</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>GET /api/v1/analytics/dashboard/academic?siteId=&amp;termId= (permiso analytics:academic:read)</t>
+          <t>core.wallet.transaction-posted.v1</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>{"siteName": "string", "quarter": "string", "previousQuarter": "string", "kpis": [{"id": "string", "label": "string", "value": "number", "unit": "string", "delta": {"value": "number", "tone": "positive | negative | neutral"}}], "subjectApprovalRates": [{"code": "string", "name": "string", "approvalRate": "number", "series": [{"quarter": "string", "approvalRate": "number"}]}], "teacherApprovalRates": [{"teacherName": "string", "subjectName": "string", "approvalRate": "number"}], "facultyTrends": [{"facultyName": "string", "points": [{"quarter": "string", "approvalRate": "number"}]}], "lastIngestionAt": "ISO 8601 UTC"} — materias en curso, tasa de aprobación por materia y por docente.</t>
+          <t>data: {"transactionId": "uuid", "userId": "uuid", "type": "CREDIT | DEBIT | REVERSAL", "concept": "TOP_UP | PAYROLL | SCHOLARSHIP | ADJUSTMENT | LIBRARY_FINE | DINING_RESERVATION | STORE_PURCHASE | EVENT_REGISTRATION | REFUND", "amount": "string decimal", "currency": "ARS", "sourceModule": "string", "externalReference": "string", "status": "POSTED"} — movimientos del mes en curso por concepto (los totales oficiales salen de aggregates). No se persiste userId.</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>{"siteName": "Todas las sedes", "quarter": "2026-1C", "previousQuarter": "2025-2C", "kpis": [{"id": "subjects-in-progress", "label": "Materias en curso", "value": 148, "unit": "materias", "delta": {"value": 6, "tone": "positive"}}], "subjectApprovalRates": [{"code": "INF-302", "name": "Desarrollo de Aplicaciones II", "approvalRate": 0.78, "series": [{"quarter": "2025-2C", "approvalRate": 0.74}, {"quarter": "2026-1C", "approvalRate": 0.78}]}], "teacherApprovalRates": [{"teacherName": "Ana Gómez", "subjectName": "Desarrollo de Aplicaciones II", "approvalRate": 0.81}], "lastIngestionAt": "2026-10-20T22:14:00.000Z"}</t>
+          <t>data: {"transactionId": "386865f7-c8aa-4aba-a374-ec9e6f8a6300", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "type": "DEBIT", "concept": "STORE_PURCHASE", "amount": "3500.00", "currency": "ARS", "sourceModule": "store", "externalReference": "purchase/93b28f67-e111-4a0d-b857-fdd015c4d3f1", "status": "POSTED"}</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>— (consumo interno: portal de Analítica)</t>
+          <t>CORE (Wallet)</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Salida</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Restful API</t>
+          <t>Message Queue</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>GET /api/v1/analytics/dashboard/financial?siteId=&amp;month=AAAA-MM (permiso analytics:finance:read)</t>
+          <t>core.wallet.transaction-rejected.v1</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>{"siteName": "string", "month": "string", "kpis": ["KpiCard"], "monthlyBalance": [{"month": "string", "income": "string decimal", "expense": "string decimal", "result": "string decimal", "balance": "string decimal"}], "administrativeExpenses": [{"category": "string", "amount": "string decimal", "percentage": "number"}], "topSellingProducts": [{"productName": "string", "category": "string", "unitsSold": "number", "revenue": "string decimal"}], "diningRevenues": [{"siteName": "string", "revenue": "string decimal", "ticketsCount": "number", "averageTicket": "string decimal"}], "lastIngestionAt": "ISO 8601 UTC"} — balances de saldo, gastos administrativos (sueldos), productos más vendidos y facturación de comedores por sede.</t>
+          <t>data: {"userId": "uuid", "type": "string", "concept": "string", "amount": "string decimal", "currency": "ARS", "sourceModule": "string", "externalReference": "string", "reasonCode": "string"} — cobros rechazados por concepto (p. ej. saldo insuficiente). Informativo.</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>{"siteName": "Sede Monserrat", "month": "2026-08", "monthlyBalance": [{"month": "2026-08", "income": "4210500.00", "expense": "10080000.00", "result": "-5869500.00", "balance": "8452300.00"}], "administrativeExpenses": [{"category": "Sueldos (PAYROLL)", "amount": "10080000.00", "percentage": 1}], "topSellingProducts": [{"productName": "Buzo UADE azul", "category": "Indumentaria", "unitsSold": 212, "revenue": "742000.00"}], "diningRevenues": [{"siteName": "Sede Monserrat", "revenue": "186000.00", "ticketsCount": 124, "averageTicket": "1500.00"}]}</t>
+          <t>data: {"userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "type": "DEBIT", "concept": "DINING_RESERVATION", "amount": "1500.00", "currency": "ARS", "sourceModule": "dining", "externalReference": "reservation/58df9fe3-4883-4dca-9d9f-4770c81543cf", "reasonCode": "WALLET_INSUFFICIENT_FUNDS"}</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>— (consumo interno: portal de Analítica)</t>
+          <t>CORE (Wallet)</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Salida</t>
+          <t>Entrada</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Restful API</t>
+          <t>Message Queue</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>GET /api/v1/analytics/events/stats?siteId=&amp;month=AAAA-MM (permiso analytics:academic:read)</t>
+          <t>core.wallet.transaction-reversed.v1</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>{"siteName": "string", "month": "string", "totalEvents": "number", "totalRegistered": "number", "totalAttendees": "number", "averageAttendanceRate": "number", "capacityOccupancy": "number", "monthlySeries": [{"month": "string", "eventsCount": "number", "attendeesCount": "number", "attendanceRate": "number"}], "lastIngestionAt": "ISO 8601 UTC"} — frecuencia, concurrencia, presentismo y ocupación de cupo.</t>
+          <t>data: {"transactionId": "uuid", "originalTransactionId": "uuid", "userId": "uuid", "concept": "REFUND", "amount": "string decimal", "currency": "ARS"} — reintegros: restitución de reservas de comedor asistidas y reversas de cobros de Tienda y Eventos.</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>{"siteName": "Sede Monserrat", "month": "2026-10", "totalEvents": 9, "totalRegistered": 640, "totalAttendees": 512, "averageAttendanceRate": 0.8, "capacityOccupancy": 0.71, "monthlySeries": [{"month": "2026-10", "eventsCount": 9, "attendeesCount": 512, "attendanceRate": 0.8}]}</t>
+          <t>data: {"transactionId": "0c3b6d21-9a44-4f7d-b2e8-15ac9f3d7e60", "originalTransactionId": "386865f7-c8aa-4aba-a374-ec9e6f8a6300", "userId": "ba310c57-a684-4dbf-a4a4-905fcfbefa08", "concept": "REFUND", "amount": "1500.00", "currency": "ARS"}</t>
         </is>
       </c>
     </row>
@@ -1538,54 +1538,150 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>GET /api/v1/analytics/filters</t>
+          <t>GET /api/v1/analytics/dashboard/academic?siteId=&amp;termId= (permiso analytics:academic:read)</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>{"sites": [{"siteId": "uuid", "code": "string", "name": "string"}], "terms": [{"termId": "uuid", "label": "string", "startDate": "date", "endDate": "date"}], "months": ["AAAA-MM"], "defaults": {"siteId": "uuid | null", "termId": "uuid", "month": "AAAA-MM"}} — opciones de filtros: sedes de Backoffice, cuatrimestres de Gestión Académica y meses con datos.</t>
+          <t>{"siteName": "string", "quarter": "string", "previousQuarter": "string", "kpis": [{"id": "string", "label": "string", "value": "number", "unit": "string", "delta": {"value": "number", "tone": "positive | negative | neutral"}}], "subjectApprovalRates": [{"code": "string", "name": "string", "approvalRate": "number", "series": [{"quarter": "string", "approvalRate": "number"}]}], "teacherApprovalRates": [{"teacherName": "string", "subjectName": "string", "approvalRate": "number"}], "facultyTrends": [{"facultyName": "string", "points": [{"quarter": "string", "approvalRate": "number"}]}], "lastIngestionAt": "ISO 8601 UTC"} — materias en curso, tasa de aprobación por materia y por docente.</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>{"sites": [{"siteId": "3e9b0a12-55cc-4d77-9a01-6b2f8c4e1d90", "code": "MONSERRAT", "name": "Sede Monserrat"}], "terms": [{"termId": "d4e5f6a7-b8c9-4d0e-9f1a-2b3c4d5e6f70", "label": "2026-2C", "startDate": "2026-08-10", "endDate": "2026-12-12"}], "months": ["2026-08", "2026-09", "2026-10"], "defaults": {"siteId": null, "termId": "d4e5f6a7-b8c9-4d0e-9f1a-2b3c4d5e6f70", "month": "2026-10"}}</t>
+          <t>{"siteName": "Todas las sedes", "quarter": "2026-1C", "previousQuarter": "2025-2C", "kpis": [{"id": "subjects-in-progress", "label": "Materias en curso", "value": 148, "unit": "materias", "delta": {"value": 6, "tone": "positive"}}], "subjectApprovalRates": [{"code": "INF-302", "name": "Desarrollo de Aplicaciones II", "approvalRate": 0.78, "series": [{"quarter": "2025-2C", "approvalRate": 0.74}, {"quarter": "2026-1C", "approvalRate": 0.78}]}], "teacherApprovalRates": [{"teacherName": "Ana Gómez", "subjectName": "Desarrollo de Aplicaciones II", "approvalRate": 0.81}], "lastIngestionAt": "2026-10-20T22:14:00.000Z"}</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
+          <t>— (consumo interno: portal de Analítica)</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Restful API</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>GET /api/v1/analytics/dashboard/financial?siteId=&amp;month=AAAA-MM (permiso analytics:finance:read)</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>{"siteName": "string", "month": "string", "kpis": ["KpiCard"], "monthlyBalance": [{"month": "string", "income": "string decimal", "expense": "string decimal", "result": "string decimal", "balance": "string decimal"}], "administrativeExpenses": [{"category": "string", "amount": "string decimal", "percentage": "number"}], "topSellingProducts": [{"productName": "string", "category": "string", "unitsSold": "number", "revenue": "string decimal"}], "diningRevenues": [{"siteName": "string", "revenue": "string decimal", "ticketsCount": "number", "averageTicket": "string decimal"}], "lastIngestionAt": "ISO 8601 UTC"} — balances de saldo, gastos administrativos (sueldos), productos más vendidos y facturación de comedores por sede.</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>{"siteName": "Sede Monserrat", "month": "2026-08", "monthlyBalance": [{"month": "2026-08", "income": "4210500.00", "expense": "10080000.00", "result": "-5869500.00", "balance": "8452300.00"}], "administrativeExpenses": [{"category": "Sueldos (PAYROLL)", "amount": "10080000.00", "percentage": 1}], "topSellingProducts": [{"productName": "Buzo UADE azul", "category": "Indumentaria", "unitsSold": 212, "revenue": "742000.00"}], "diningRevenues": [{"siteName": "Sede Monserrat", "revenue": "186000.00", "ticketsCount": 124, "averageTicket": "1500.00"}]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>— (consumo interno: portal de Analítica)</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Restful API</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>GET /api/v1/analytics/events/stats?siteId=&amp;month=AAAA-MM (permiso analytics:academic:read)</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>{"siteName": "string", "month": "string", "totalEvents": "number", "totalRegistered": "number", "totalAttendees": "number", "averageAttendanceRate": "number", "capacityOccupancy": "number", "monthlySeries": [{"month": "string", "eventsCount": "number", "attendeesCount": "number", "attendanceRate": "number"}], "lastIngestionAt": "ISO 8601 UTC"} — frecuencia, concurrencia, presentismo y ocupación de cupo.</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>{"siteName": "Sede Monserrat", "month": "2026-10", "totalEvents": 9, "totalRegistered": 640, "totalAttendees": 512, "averageAttendanceRate": 0.8, "capacityOccupancy": 0.71, "monthlySeries": [{"month": "2026-10", "eventsCount": 9, "attendeesCount": 512, "attendanceRate": 0.8}]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>— (consumo interno: portal de Analítica)</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Restful API</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>GET /api/v1/analytics/filters</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>{"sites": [{"siteId": "uuid", "code": "string", "name": "string"}], "terms": [{"termId": "uuid", "label": "string", "startDate": "date", "endDate": "date"}], "months": ["AAAA-MM"], "defaults": {"siteId": "uuid | null", "termId": "uuid", "month": "AAAA-MM"}} — opciones de filtros: sedes de Backoffice, cuatrimestres de Gestión Académica y meses con datos.</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>{"sites": [{"siteId": "3e9b0a12-55cc-4d77-9a01-6b2f8c4e1d90", "code": "MONSERRAT", "name": "Sede Monserrat"}], "terms": [{"termId": "d4e5f6a7-b8c9-4d0e-9f1a-2b3c4d5e6f70", "label": "2026-2C", "startDate": "2026-08-10", "endDate": "2026-12-12"}], "months": ["2026-08", "2026-09", "2026-10"], "defaults": {"siteId": null, "termId": "d4e5f6a7-b8c9-4d0e-9f1a-2b3c4d5e6f70", "month": "2026-10"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
           <t>CORE (Gateway)</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>Salida</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>Restful API</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Restful API</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>GET /health/live · GET /health/ready</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>Res 200: {"status": "string", "checks": {"db": "string", "broker": "string"}}</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="F40" s="5" t="inlineStr">
         <is>
           <t>{"status": "ok", "checks": {"db": "up", "broker": "up"}}</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F37"/>
+  <autoFilter ref="A4:F40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>